<commit_message>
docs: add partial answer for week 4
</commit_message>
<xml_diff>
--- a/raw_csv_quiz/Quiz_Week04.xlsx
+++ b/raw_csv_quiz/Quiz_Week04.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\LearningHub\ai-2y-journey\06-other\flashcard-app\raw_csv_quiz\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C88F6DE-9F20-474D-88AF-125276EAC4D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CE04C0E-3896-4444-963E-C6BC15CB9DF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2988" yWindow="792" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Questions" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1066" uniqueCount="680">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1098" uniqueCount="712">
   <si>
     <t>Question</t>
   </si>
@@ -2173,6 +2173,308 @@
 IAM User (Option A): You give a contractor a Permanent ID Card and a physical key to the front door. If they lose it, anyone can walk in forever until you change the locks.
 IAM Role (Option B): You give the contractor a Temporary Visitor Badge. It only works for the 8 hours they are scheduled to work. At the end of the day, the badge automatically deactivates. This is much safer!
 Key Exam Keyword: Whenever you see "No long-term credentials," "EC2 to S3," or "Safest way for instances," the answer is always IAM Role.</t>
+  </si>
+  <si>
+    <t>D. Enterprise Support.
+Why is this the answer?
+While several AWS support plans offer technical assistance, the specific requirements listed—especially the Technical Account Manager (TAM) and the 15-minute response time—are exclusive "markers" for the Enterprise tier.
+The Technical Account Manager (TAM): This is the biggest giveaway. A TAM is a dedicated primary point of contact who provides architectural guidance, cost optimization, and operational reviews. They are only included in the Enterprise and Enterprise On-Ramp plans (though Enterprise provides a dedicated TAM).
+15-Minute Response Time: For "Business-Critical System Down" cases, Enterprise Support guarantees a response from a senior engineer within 15 minutes. For comparison, the Business plan's fastest response is 1 hour for "Urgent" cases.
+Full Trusted Advisor Checks: While the Business plan also provides access to all Trusted Advisor checks, only the Enterprise plan includes prioritized recommendations and deep-dive reviews led by your dedicated account team (TAM and Solution Architects).
+Why the other options are wrong:
+A. Basic Support: This is the free tier. It includes no technical support and only a handful of "core" Trusted Advisor checks.
+B. Developer Support: This provides "Business hour" access to support via email for a single primary contact. It does not include 24/7 phone support, a TAM, or any "System Down" response priority.
+C. Business Support: This is a popular tier for production workloads as it offers 24/7 support and the full set of Trusted Advisor checks. However, it lacks a TAM and its fastest response time is 1 hour, not 15 minutes.</t>
+  </si>
+  <si>
+    <t>Think of AWS Support levels like staying at a hotel:
+Basic: You stay for free, but there is no staff. You have to find your own towels and fix the sink yourself using a manual.
+Developer: There is a front desk clerk available during the day, but they only respond to messages left under the door.
+Business: There is a 24/7 front desk. If your toilet overflows, they'll send someone within an hour.
+Enterprise: You have a Private Concierge (The TAM). They know your preferences, they help you plan your entire trip (Architecture), and if there is a life-threatening emergency, they are at your door in 15 minutes. (This Answer)
+Key Exam Keyword: Whenever you see "TAM," "Technical Account Manager," or "15-minute response," the answer is always Enterprise Support.</t>
+  </si>
+  <si>
+    <t>C. Use the consolidated billing feature from AWS Organizations.
+Why is this the answer?
+AWS rewards customers who spend more by lowering the "unit price" of services like S3 storage or Data Transfer. However, if your spending is split across ten small accounts, you might not hit the high-volume tiers in any of them.
+Volume Discounts: AWS looks at the total usage of all accounts in the organization as if they were one single account. This helps you reach lower-priced tiers (volume discounts) much faster.
+Minimal Impact: This is a billing-only change. You do not have to move servers, change IP addresses, or shut down any resources. The accounts simply become "members" of an organization.
+One Bill: You get one consolidated invoice for all accounts, making life much easier for the accounting department.
+Shared Savings: If one account purchases a Savings Plan or Reserved Instance but doesn't use it all, the discount can "float" and be applied to a different account within the same Organization.
+Why the other options are wrong:
+A. One global account: This is the opposite of "minimal impact." Moving resources between accounts is a massive technical project that involves downtime, reconfiguration, and risk. It’s better to keep the accounts separate for security but join them for billing.
+B. Three years of Reserved Instances: While this provides a discount, it is a commitment for specific resources. It doesn't automatically give you volume discounts on things like S3 storage or data transfer across your entire company.
+D. Enterprise Support: This is a high-cost service plan for technical help. While Enterprise customers might have custom "Enterprise Agreements," simply signing up for the support plan does not automatically trigger the standard volume discounts that Consolidated Billing provides.</t>
+  </si>
+  <si>
+    <t>Think of your AWS accounts like members of a family with cell phones:
+Separate Billing: Every person has their own 5GB plan. If Mom uses 1GB and Son uses 9GB, Mom pays for 5GB (wasted) and Son pays huge "overage" fees.
+Consolidated Billing (The Answer): You put everyone on one Family Plan. The carrier looks at the total usage (10GB). Because you are buying in bulk, the "price per GB" drops, and if Mom doesn't use her data, Son can use it without extra fees. No one had to change their phone number or buy a new phone (Minimal Impact).
+Key Exam Keyword: Whenever you see "Multiple accounts," "Volume discounts," or "Consolidated billing," the answer is AWS Organizations.</t>
+  </si>
+  <si>
+    <t>C. AWS Budgets.
+Why is this the answer?
+While several tools help you look at your money, AWS Budgets is the specific tool designed for proactive alerting based on limits you define.
+Custom Thresholds: You can set a budget for a specific dollar amount (e.g., "$100 per month") or a usage amount (e.g., "2,000 hours of EC2 usage").
+Actual vs. Forecasted: This is a "killer feature." You can set an alert to trigger if your actual spend hits 80%, OR if AWS forecasts that you are on track to exceed your budget by the end of the month.
+Notification Integration: It integrates directly with SNS (Simple Notification Service) and Email. This means you can get a text message, an email, or even trigger an automated "Lambda" function to shut down servers if a budget is exceeded.
+Why the other options are wrong:
+A. AWS Cost Explorer: This is a visualization tool. It's great for looking at graphs and seeing where your money went last month, but it doesn't "watch" your account and send emails when a limit is hit.
+B. AWS Trusted Advisor: This is a best-practice tool. It will tell you if you have "idle" resources that are wasting money, but it isn't the primary tool for setting specific dollar-amount alerts.
+C. AWS Cost Anomaly Detection: This uses machine learning to find unusual spending patterns (e.g., a sudden $200 spike in a service you never use). While it sends alerts, it doesn't work based on a "predefined threshold" that you set; it works based on what the AI thinks is "weird."</t>
+  </si>
+  <si>
+    <t>Think of your AWS spending like a Car Trip:
+AWS Cost Explorer: This is like looking at your Receipt after you finish the trip to see how much you spent on gas.
+AWS Cost Anomaly Detection: This is like a Warning Light that turns on if your engine is acting strange.
+AWS Budgets (The Answer): This is like setting a GPS Alert that pings your phone every time you've spent another $20 on gas, or warns you: "Based on your speed, you will run out of money before you reach your destination."
+Key Exam Keyword: Whenever you see "Custom Alerts," "Notify via Email/SNS," or "Exceeds Threshold," the answer is AWS Budgets.</t>
+  </si>
+  <si>
+    <t>D. Spot Instances.
+Why is this the answer?
+AWS Spot Instances are designed exactly for this scenario: high-scale computing at the lowest possible cost.Spare Capacity: AWS has massive data centers. Not every server is being used at 100% capacity all the time. Spot Instances allow you to "bid" on this unused capacity.Deepest Discounts: Because this is "surplus" inventory, AWS offers it at a massive discount—up to 90% off the On-Demand price.The "Trade-off" (Interruptions): The catch is that AWS can reclaim these instances with only a two-minute notice if they need the capacity back for full-paying On-Demand customers.Perfect Use Case: Since your workload is a batch processing job that can be interrupted and resumed, it is the perfect candidate. If AWS takes the server away, your job simply waits for a new Spot Instance to become available and picks up where it left off (or restarts the batch).Why the other options are wrong:A &amp; C. Reserved Instances (Standard/Convertible): These offer significant discounts (up to 72%), but they require a 1 or 3-year commitment. They are intended for "Steady State" workloads that run 24/7, not short-term batch jobs.B. On-Demand Instances: These are the most expensive. You pay the full "sticker price" for the benefit of never being interrupted. Since your job can be interrupted, using On-Demand would be a waste of money.</t>
+  </si>
+  <si>
+    <t>Think of Spot Instances like Standby Airfare:
+On-Demand (Option B): You buy a Full-Price Ticket. You are guaranteed a seat, and the airline won't kick you off the plane.
+Reserved Instances (Options A/C): You buy a 3-Year Season Pass. It's cheaper per flight, but you're committed to flying with that airline for a long time.
+Spot Instances (The Answer): You buy a Standby Ticket. It is 90% cheaper, but you only get to fly if there's an empty seat. If a full-price passenger shows up at the last minute, you have to get off the plane and wait for the next one. (This Answer)
+Key Exam Keyword: Whenever you see "Deepest discount," "Up to 90%," or "Fault-tolerant/Interruption-tolerant," the answer is always Spot Instances.</t>
+  </si>
+  <si>
+    <t>C. Each AWS account gets volume discounts.
+Why is this the answer?
+AWS rewards customers who use more services by lowering the "price per unit." However, if your usage is spread across five separate accounts, you might not be hitting the high-usage thresholds in any of them individually.
+Combined Usage: When you set up Consolidated Billing (via AWS Organizations), AWS treats all the accounts as a single account for billing purposes.
+Faster Tiering: If Account A uses 4 TB of S3 storage and Account B uses 7 TB, AWS sees a total of 11 TB. Since S3 prices often drop after the first 10 TB, the accounts collectively reach that "lower-priced tier" much faster.
+Shared Savings: Beyond volume discounts, accounts also share the benefits of Reserved Instances (RIs) and Savings Plans. If one account has an unused RI, that discount can automatically "float" to another account in the organization to save money.
+Why the other options are wrong:
+A. Costs reduced to half: While you save money through volume discounts, AWS does not simply slash your bill by 50% just for turning on a feature. Savings depend entirely on your usage levels.
+B. Just for organizational purpose: While it definitely helps with organization (one invoice instead of five!), its primary financial benefit is cost reduction through aggregated usage.
+D. Five times the free-tier capacity: This is a common trap! In fact, it's the opposite. When you consolidate accounts, they all share a single account's worth of Free Tier benefits. You don't get five times the free hours; you get one pool that all five accounts pull from.</t>
+  </si>
+  <si>
+    <t>Think of your five AWS accounts like five neighbors:
+Separate Billing: Each neighbor goes to the grocery store and buys a small 1L bottle of water. They all pay the high "single-bottle" price.
+Consolidated Billing (The Answer): One neighbor (the Master/Management Account) goes to a warehouse club and buys a 50-pack case of water for everyone. Because they bought in bulk, the "price per bottle" is much lower for everyone. (This Answer)
+Key Exam Keyword: Whenever you see "Multiple accounts" and "Volume discounts," the answer is Consolidated Billing.</t>
+  </si>
+  <si>
+    <t>D. AWS Secrets Manager.
+Why is this the answer?
+This question highlights the specific difference between a service that manages secrets and a service that simply encrypts data.
+Secret Rotation: This is the "killer feature" of AWS Secrets Manager. It can automatically change (rotate) passwords for services like Amazon RDS, Redshift, and DocumentDB without you having to write complex code or manually update a config file.
+Secure Storage: It stores credentials (like database passwords, API keys, and OAuth tokens) in an encrypted format.
+Programmatic Retrieval: Instead of hardcoding a password in your application code, your code calls the Secrets Manager API to "get the secret." This keeps your code clean and secure.
+KMS Integration: Secrets Manager actually uses AWS KMS behind the scenes to encrypt the password, but Secrets Manager provides the "wrapper" that handles the logic of rotation and retrieval.
+Why the other options are wrong:
+A. AWS KMS: While KMS is used for encrypting data (like S3 buckets or EBS volumes), it does not have the built-in logic to "log into a database and change the password." It provides the "locks," but not the "management."
+B. AWS IAM: This is for Identity and Access Management. You use it to create users, groups, and roles. It does not store third-party credentials (like a GitHub API key) or handle automatic password rotation for databases.
+C. AWS Artifact: This is a "document portal." You use it to download compliance reports (like ISO or SOC reports) to prove to auditors that AWS is secure. It has nothing to do with passwords or encryption.</t>
+  </si>
+  <si>
+    <t>Think of your security setup like a high-end hotel:
+AWS KMS: This is the Master Key. It’s the tool used to lock and unlock doors, but it doesn't care what is inside the room.
+AWS Secrets Manager (The Answer): This is the Digital Safe inside the hotel room. It holds the valuables (the passwords). Best of all, it has a feature where it automatically changes its own combination every 30 days so that even if an old code is stolen, it won't work anymore.
+Key Exam Keyword: Whenever you see "Rotate credentials," "Database passwords," or "API keys," the answer is AWS Secrets Manager.</t>
+  </si>
+  <si>
+    <t>B. The IAM user does not have an IAM policy attached that explicitly grants them S3 permissions.
+Why is this the answer?
+This question tests your understanding of the "Intersection of Permissions" within AWS Organizations. To perform an action in a member account, a user needs two green lights: one from the Organization (the SCP) and one from the Account (the IAM Policy).
+SCPs are "Guardrails," not "Givers": A Service Control Policy (SCP) sets the maximum permissions for an account. If an SCP allows S3, it doesn't mean everyone in the account suddenly has S3 access; it simply means S3 is permitted to be used within that account.
+The IAM Requirement: Within the member account, the administrator still needs to create an IAM policy (Identity-based policy) and attach it to the user. Without that IAM policy, the default state of AWS is "Deny Everything."
+The Logical "AND": Think of it as a logical AND gate.
+(SCP allows S3) AND (IAM Policy allows S3) = Access Granted.
+(SCP allows S3) AND (No IAM Policy) = Access Denied.
+Why the other options are wrong:
+A. SCPs only monitor billing: This is incorrect. SCPs are a security feature used for access control, not a billing tool. You are likely thinking of AWS Budgets or Consolidated Billing.
+C. Master account must perform action: There is no "activation" required. Once an SCP is attached to an OU or account, it is active immediately.
+D. Applied directly to the user: SCPs cannot be attached to individual IAM users. They can only be attached to the Root of the organization, Organizational Units (OUs), or Member Accounts.</t>
+  </si>
+  <si>
+    <t>Imagine you are trying to enter a specific country (Amazon S3):
+The SCP (Option B): This is like the Diplomatic Agreement between your home country and the destination. If the agreement says "People from your country are allowed to visit," the border is open. But the agreement itself isn't your travel document.
+The IAM Policy: This is your Personal Visa. Even if the countries are friendly (the SCP allows it), the border guard will turn you away if you don't have your own visa in your hand. (This Answer)
+Key Exam Keyword: Whenever you see a scenario where an SCP allows something but the user is Denied, check if the user has an IAM Policy. The SCP is the "Boundary," and the IAM Policy is the "Permission."</t>
+  </si>
+  <si>
+    <t>B. Invisible costs like uncleaned storage and unmodeled data transfer.
+Why is this the answer?
+According to various cloud financial management (FinOps) studies and AWS "Value Gap" reports, the majority of budget overruns in AI and large-scale projects aren't caused by the servers themselves, but by the "waste" that accumulates around them.
+Orphaned Resources: When data scientists spin up powerful GPU instances to train a model, they often create EBS (Elastic Block Store) volumes for storage. If they delete the instance but forget to check the box to "Delete on Termination," that storage stays active and continues to bill you indefinitely—even though it's not attached to anything.
+Unmodeled Data Transfer: Moving data between AWS Regions or even between different Availability Zones (AZs) carries a cost. AI workloads often involve moving massive datasets ($150+$ petabytes in some case studies) for training. If these "egress" or "cross-zone" costs aren't included in the initial architecture model, they create a massive "invisible" bill at the end of the month.
+The "Safety Buffer" Trap: Engineering teams often over-provision resources by $30\% - 40\%$ "just to be safe" during model training. This idle capacity is a primary driver of the observed budget gaps in mid-to-large-sized AI projects.
+Why the other options are wrong:
+A. Rapid scaling of On-Demand: While expensive, scaling is usually visible and expected during growth. The "budget gap" specifically refers to the difference between what teams thought they would spend and what they actually spent due to things they missed.
+C. High premium charges for Support: Support plans are fixed percentages or flat fees. They are very predictable and rarely the cause of a "gap" or surprise.
+D. Inaccurate pricing forecasts: The AWS Cost Explorer is actually quite accurate; the "inaccuracy" usually comes from humans failing to input all variables (like data transfer) into the calculation, rather than the tool itself being broken.</t>
+  </si>
+  <si>
+    <t>Think of your AWS bill like your home's energy bill:
+On-Demand Instances (Option A): These are like your Lights and Air Conditioning. You know when they are on, and you expect to pay for them.
+Invisible Costs (The Answer): These are like "Ghost" appliances—the old refrigerator in the garage you forgot to unplug, or the heater running in a room with the windows open. You don't "see" them working, but they are the reason your bill is $\$200$ higher than you calculated. (This Answer)Key Exam Keyword: Whenever a question asks about "Unexpected spend" or "Budget gaps," look for words like "Unattached/Orphaned EBS," "Idle resources," or "Data Transfer."</t>
+  </si>
+  <si>
+    <t>B. Amazon GuardDuty fits best.
+Why is this the answer?
+Amazon GuardDuty is a threat detection service that acts like a 24/7 security guard for your entire AWS infrastructure.
+Monitors Log Sources: It doesn't require you to install anything. It automatically analyzes billions of events from AWS CloudTrail (API calls), VPC Flow Logs (network traffic), and DNS Logs (queries to malicious domains).
+Intelligent Detection: It uses machine learning, anomaly detection, and integrated "threat intelligence" (lists of known bad IP addresses and domains) to identify threats.
+Specific Findings: It can detect things like:
+Unusual API calls: Someone trying to disable logging or delete backups.
+Suspicious network activity: An EC2 instance talking to a "Command and Control" server used by hackers.
+DNS-related signs: Instances using "DNS tunneling" to steal data.
+Why the other options are wrong:
+A. Amazon Macie: This is for data privacy. It scans S3 buckets to find sensitive information like credit card numbers or PII. It does not monitor network traffic or API behavior.
+C. AWS Secrets Manager: This is a vault for passwords and API keys. It handles rotation and storage but doesn't "watch" for hackers.
+D. Amazon Inspector: This is a vulnerability scanner. It looks at your EC2 instances and container images to see if you have "holes" in your software (like unpatched versions), but it doesn't monitor real-time traffic or API calls.</t>
+  </si>
+  <si>
+    <t>Think of your AWS account like a high-end office building:
+Amazon Inspector: The Building Inspector. They walk around checking if the fire extinguishers are expired or if a window is accidentally left unlocked.
+Amazon Macie: The Privacy Officer. They look inside filing cabinets to make sure you aren't leaving sensitive customer files out on the desks.
+Amazon GuardDuty (The Answer): The Security Guard. They watch the security cameras (logs) and alert you immediately if they see someone wearing a mask trying to pick a lock or if a computer in the lobby starts sending weird data to a foreign country. (This Answer)
+Key Exam Keyword: Whenever you see "Malicious activity," "Anomalous behavior," or "Monitoring DNS/VPC/CloudTrail logs" for security threats, the answer is Amazon GuardDuty.</t>
+  </si>
+  <si>
+    <t>C. It improves availability and distributes traffic across targets.
+Why is this the answer?
+This design is the standard "Best Practice" for a secure and highly available web application on AWS.
+High Availability (Multi-AZ): By deploying the Application Load Balancer (ALB) across two or more Availability Zones (AZs), you ensure that if one data center fails (due to power loss, flooding, etc.), the load balancer can still receive traffic in the other healthy zone.
+Traffic Distribution: The ALB acts as a "traffic cop." It receives a single request from the internet and distributes it among your various web servers. If one server becomes unhealthy, the ALB automatically stops sending traffic to it and reroutes those requests to the remaining healthy servers.
+Security via Isolation: The web servers are kept in private subnets, meaning they do not have public IP addresses and cannot be reached directly from the internet. The ALB sits in the public subnets to accept requests and then "reaches back" to the private servers to deliver them. This creates a powerful layer of security.
+Why the other options are wrong:
+A. Eliminates Security Groups: Incorrect. You actually need more specific Security Groups. You need one for the ALB (allowing port 80/443 from the world) and one for the EC2 instances (allowing traffic only from the ALB’s Security Group).
+B. Direct internet access for private instances: Incorrect. To give private instances direct internet access (e.g., for downloading software updates), you would need a NAT Gateway. The ALB only handles incoming requests from users to the app.
+C. Replaces Route 53: Incorrect. Route 53 (DNS) and the ALB work together. Route 53 directs the user's browser to the ALB’s DNS name (e.g., my-load-balancer-123.aws.com).</t>
+  </si>
+  <si>
+    <t>Think of your application like a VIP Club:
+The Public Subnets (The Sidewalk): This is where people line up. It's visible to the public.
+The ALB (The Bouncer): The bouncer stands at the door. He checks IDs (health checks) and tells people which room to go to. If one room is too full or "closed for cleaning," he sends people to the other room.
+The Private Subnets (The VIP Rooms): These rooms are deep inside the building. There are no windows to the street. The only way to get in is if the Bouncer (ALB) personally opens the door and lets you through.
+Key Exam Keyword: Whenever you see "Load Balancer," "Multi-AZ," or "Public/Private Subnets," the goal is Availability, Scalability, and Security.</t>
+  </si>
+  <si>
+    <t>B. AWS Security Hub &amp; Amazon EventBridge.
+Why is this the answer?
+Amazon Inspector is an automated vulnerability management service. However, it doesn't just display findings in its own console; it is designed to feed that data into other services for centralized management and automation.
+AWS Security Hub: This is the primary integration point. When you enable Security Hub, Inspector automatically sends all findings there. This allows you to see your software vulnerabilities (Inspector) alongside your threat detections (GuardDuty) and data privacy alerts (Macie) in one single dashboard.
+Amazon EventBridge: This is the "automation engine." Every time Inspector finds a new vulnerability, it publishes an event to EventBridge. You can set up rules in EventBridge to "listen" for these findings and trigger actions, such as sending a Slack notification, creating a Jira ticket, or even running an AWS Lambda function to automatically patch a server.
+Why the other options are wrong:
+A. Amazon S3 &amp; Amazon DynamoDB: While you can export reports to S3, these are not the primary services for "sending findings" for real-time security monitoring or action. DynamoDB is a database and has no native "finding ingestion" feature from Inspector.
+C. Amazon RDS &amp; AWS Lambda: Inspector can scan the OS of an EC2 instance that might be hosting a database, but it doesn't send findings to RDS. While EventBridge can trigger a Lambda function based on a finding, Inspector doesn't send findings directly to Lambda.
+D. Amazon CloudFront &amp; AWS Shield: These are edge security services. They don't have a mechanism to ingest or display vulnerability findings from Inspector.</t>
+  </si>
+  <si>
+    <t>Think of your AWS account like a high-tech building:
+Amazon Inspector: The Maintenance Worker who walks around checking every pipe and wire for leaks or frayed edges (vulnerabilities).
+AWS Security Hub (Option B): The Control Room. The maintenance worker calls the control room to report every leak so the manager can see the whole building's status on one big screen. (This Answer)
+Amazon EventBridge (Option B): The Automatic Alarm System. When the maintenance worker finds a "leak," EventBridge automatically rings a bell, turns on a light, or calls a plumber to fix it. (This Answer)
+Key Exam Keyword: Whenever you see "Send findings," "Centralized security," or "Automate responses," look for Security Hub and EventBridge.</t>
+  </si>
+  <si>
+    <t>D. AWS ACM (AWS Certificate Manager).
+Why is this the answer?
+AWS Certificate Manager (ACM) is the specific service designed to handle the complexity of creating, managing, and deploying SSL/TLS certificates.
+Provisioning: You can request a new certificate directly from AWS (issued by Amazon's own Certificate Authority) or import one you bought from a third party.
+Easy Deployment: Once a certificate is created in ACM, you can "attach" it to other AWS services like an Application Load Balancer (ALB), Amazon CloudFront, or API Gateway with just a few clicks.
+Automatic Renewal: This is the best feature. If you use certificates provided by Amazon and they are currently in use by an AWS service, ACM handles the renewal process automatically. This prevents the "expired certificate" errors that often crash websites.
+Cost: Public SSL/TLS certificates requested through ACM are free to use with integrated AWS services.
+Why the other options are wrong:
+A. Amazon GuardDuty: This is a threat detection service (the "Security Guard"). It watches your logs for hackers but doesn't handle website certificates.
+B. Amazon Detective: This is used for security investigations. If GuardDuty finds a threat, you use Detective to find the root cause. It doesn't manage SSL.
+C. AWS WAF (Web Application Firewall): This service protects your website from common web exploits (like SQL injection). While a WAF is often used alongside an SSL certificate, it doesn't provide or manage the certificate itself.</t>
+  </si>
+  <si>
+    <t>Think of your website as a building and your SSL certificate as the Building's Official ID Card:
+The ID Card (The SSL Certificate): It proves to the world that your building (website) is legitimate and that any "conversations" held inside are private (encrypted).
+AWS ACM (The Answer): This is the ID Card Office. They print the card for you, make sure it’s valid, and automatically send you a new one before the old one expires so you never have to stand in line or worry about it. (This Answer)
+Key Exam Keyword: Whenever you see "SSL/TLS," "HTTPS," or "Renewing certificates," the answer is always ACM.</t>
+  </si>
+  <si>
+    <t>C. Switch from real-time SageMaker endpoints to Batch Inference (Batch transform jobs).
+Why is this the answer?
+For AI and machine learning workloads that are non-customer-facing (meaning they don't need a response in milliseconds), real-time hosting is often a massive waste of money.
+Idle Cost Elimination: Real-time endpoints (Option A) keep a server running 24/7, waiting for a request. If you are only processing documents or forecasting demand once a day, you are paying for hours of "idle" time.
+The Batch Advantage: Batch Transform jobs spin up compute resources only when they are needed, process all your data at once, and then immediately shut down. You only pay for the exact minutes the processing takes.
+Significant Savings: This shift typically results in the 60-70% cost reduction mentioned in the prompt because it removes the "always-on" overhead.
+Fit for Purpose: Document processing (OCR) and demand forecasting are "asynchronous" tasks. The user doesn't need the result immediately, making them perfect for batch processing.
+Why the other options are wrong:
+A. Compress vector embeddings: While HNSW (Hierarchical Navigable Small World) and Product Quantization (PQ) are great for making vector databases faster and smaller, this primarily impacts storage and latency. It doesn't address the massive compute costs of running inference servers.
+B. Set budget alerts at $5,000 increments: This is a monitoring strategy, not an optimization strategy. Furthermore, as we discussed earlier, $5,000 increments are too large for effective "early" detection of overspend.
+D. Implement Cost Allocation Tags: Tagging is essential for accountability (knowing who spent the money), but it doesn't actually reduce the bill. It just tells you who to blame for the high bill!</t>
+  </si>
+  <si>
+    <t>Think of your AI processing like doing your laundry:
+Real-time Endpoint: This is like keeping your washing machine running 24/7, even when empty, just in case you want to throw in one sock at 3:00 AM. It’s convenient, but your electricity bill will be insane.
+Batch Inference (The Answer): This is like waiting until you have a full basket of clothes and running the machine once. It uses the same amount of power to clean the clothes, but the machine is off the rest of the day, saving you a fortune. (This Answer)
+Key Exam Keyword: Whenever you see "Non-real-time," "Background processing," or "Reduce cost for ML," look for Batch Transform or Batch Inference.</t>
+  </si>
+  <si>
+    <t>In the AWS Cloud Practitioner curriculum, compute cost for services like Amazon EC2 is fundamentally calculated by looking at three main variables:
+Instance Type: This represents the "Price per Hour" (or second). Different instance types (e.g., t3.micro vs. p4d.24xlarge) have different costs based on the CPU, RAM, and hardware capabilities.
+Instance Amount: The total number of virtual servers you have running at the same time.
+Runtime: The duration the instances are in a "running" state. AWS bills EC2 by the second (with a 60-second minimum) for Linux and Windows instances.
+Multiplying these three together gives you the total bill for your compute resources.
+Why the other options are wrong:
+B. Storage × Requests × Region: This is more characteristic of Amazon S3 (Storage) or Amazon DynamoDB (Requests/Provisioned Capacity). While "Region" does affect compute pricing, it isn't a variable you multiply in a formula; it's a fixed part of the "Instance Type" rate.
+C. Runtime × Bandwidth × Users: Bandwidth (Data Transfer Out) is a separate cost driver in AWS. "Number of users" is almost never a direct billing metric for core infrastructure like EC2.
+D. Instance Type × Availability Zone × Storage: This is a mix of different billing units. Storage (EBS) is billed by GB-month, which is separate from the hourly/second compute charge for the instance itself.</t>
+  </si>
+  <si>
+    <t>Think of your compute cost like renting a fleet of cars for a road trip:Instance Type: 
+The Model of the car (A luxury SUV costs more per hour than a compact car).
+Instance Amount: How many cars you are renting at once for your group.
+Runtime: How many hours you keep the keys.
+Formula: $Price of Model * Number of Cars * Hours Used = Total Bill$
+Key Exam Keyword: When calculating EC2 cost, look for Instance Type, Count, and Time (Usage).</t>
+  </si>
+  <si>
+    <t>C. Amazon GuardDuty.
+Why is this the answer?
+Amazon GuardDuty is a threat detection service that acts as a 24/7 intelligent monitor for your entire AWS environment.
+AI &amp; Machine Learning (ML): GuardDuty doesn't just look for "known" threats. It uses advanced machine learning and anomaly detection to learn what "normal" behavior looks like for your account. If it sees something that breaks that pattern, it flags it as a potential threat.
+Continuous Monitoring: It works in the background, continuously analyzing billions of events from primary log sources without you having to install any software or agents.
+Broad Visibility: It monitors three key data sources to catch malicious activity:
+AWS CloudTrail Logs: To detect unusual API calls (e.g., someone trying to delete your backups).
+VPC Flow Logs: To spot suspicious network traffic (e.g., your server talking to a known hacker "command" server).
+DNS Logs: To identify if an instance is communicating with malicious domains.
+Why the other options are wrong:
+A. AWS Macie: While Macie does use machine learning, its primary job is data privacy. It scans your S3 buckets to find sensitive data like credit card numbers or PII. It does not monitor network traffic or API behavior for hacking threats.
+B. AWS KMS: This is a cryptography service. It manages the "keys" used to encrypt and decrypt your data. It is a tool used for protection, not a monitoring service for malicious activity.
+D. AWS CloudTrail: This is a logging service. It records every action (API call) taken in your account. While GuardDuty uses CloudTrail data to find threats, CloudTrail itself is just a "recorder"—it doesn't "monitor" or "analyze" for malicious behavior on its own.</t>
+  </si>
+  <si>
+    <t>Think of your AWS account like a high-end bank:
+AWS CloudTrail (Option D): These are the Security Cameras. They record everything that happens, but someone has to watch the tapes to find a crime.
+AWS Macie (Option A): This is the Privacy Auditor. They look inside the envelopes in the safe to make sure no one left their social security numbers out in the open.
+Amazon GuardDuty (The Answer): This is the Intelligent Security Guard. He watches the cameras in real-time, recognizes that a person in a mask is acting suspiciously (Machine Learning), and immediately sounds the alarm before the vault is even touched. (This Answer)
+Key Exam Keyword: Whenever you see "Machine Learning," "Threat Detection," or "Intelligent monitoring of logs," the answer is Amazon GuardDuty.</t>
+  </si>
+  <si>
+    <t>C. IAM Credentials Report.
+Why is this the answer?
+The IAM Credentials Report is the primary auditing tool for account-wide security hygiene regarding passwords and access keys.
+Comprehensive Data: It generates a CSV file that lists every user in your account and the status of their various credentials, including passwords, access keys, and MFA devices.
+Usage Tracking: For every access key, the report explicitly lists the "access_key_X_last_used_date". This allows a security team to easily filter the list for any key where the last used date is older than 90 days.
+Audit Readiness: It is the go-to tool for compliance audits because it provides a "snapshot" of the security state of all users at a specific point in time.
+No Cost: You can generate this report as often as once every four hours at no additional charge.
+Why the other options are wrong:
+A. IAM Access Advisor: This tool tells you which services (like S3 or EC2) a user has accessed and when. While useful for "Least Privilege" auditing, it doesn't provide a downloadable report focused specifically on the age and status of Access Keys for the entire account in one view.
+B. AWS CloudTrail: While CloudTrail records every API call, using it to find "unused" keys is extremely difficult. You would have to search through millions of logs to see which keys didn't appear, which is much more work than just running a Credentials Report.
+D. AWS Config: This service tracks configuration changes over time (e.g., "When was this S3 bucket made public?"). While it can alert you if a user is created, it isn't designed to generate a status report of credential usage dates.</t>
+  </si>
+  <si>
+    <t>Think of your AWS account like an office building:
+AWS CloudTrail (Option B): The Security Camera footage. You can see who walked through the door today, but it’s hard to tell who hasn't visited in three months just by watching tapes.
+IAM Access Advisor (Option A): The Room Logs. It shows that "User A" entered the Breakroom and the Server Room, but not the Executive Suite.
+IAM Credentials Report (The Answer): The Manager's Spreadsheet. It lists every employee and exactly when their keycard was last scanned at the front gate. If the spreadsheet says "Last Scanned: January" and it's now April, you know it's time to deactivate that card. (This Answer)
+Key Exam Keyword: Whenever you need to audit or get a list/report of all users and their credential age/last used date, the answer is IAM Credentials Report.</t>
   </si>
 </sst>
 </file>
@@ -2874,7 +3176,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>77</v>
       </c>
@@ -2893,8 +3195,14 @@
       <c r="F17" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G17" s="2" t="s">
+        <v>696</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>697</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>82</v>
       </c>
@@ -2914,7 +3222,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>87</v>
       </c>
@@ -2934,7 +3242,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>92</v>
       </c>
@@ -2954,7 +3262,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>97</v>
       </c>
@@ -2974,7 +3282,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>102</v>
       </c>
@@ -2994,7 +3302,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>107</v>
       </c>
@@ -3014,7 +3322,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>112</v>
       </c>
@@ -3034,7 +3342,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>117</v>
       </c>
@@ -3054,7 +3362,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>122</v>
       </c>
@@ -3074,7 +3382,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>124</v>
       </c>
@@ -3094,7 +3402,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>129</v>
       </c>
@@ -3113,8 +3421,14 @@
       <c r="F28" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G28" s="2" t="s">
+        <v>706</v>
+      </c>
+      <c r="H28" s="2" t="s">
+        <v>707</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>134</v>
       </c>
@@ -3134,7 +3448,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>139</v>
       </c>
@@ -3154,7 +3468,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>144</v>
       </c>
@@ -3174,7 +3488,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>149</v>
       </c>
@@ -3420,7 +3734,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>197</v>
       </c>
@@ -3438,6 +3752,12 @@
       </c>
       <c r="F44" t="s">
         <v>22</v>
+      </c>
+      <c r="G44" s="2" t="s">
+        <v>698</v>
+      </c>
+      <c r="H44" s="2" t="s">
+        <v>699</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.3">
@@ -3666,7 +3986,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>240</v>
       </c>
@@ -3684,6 +4004,12 @@
       </c>
       <c r="F56" t="s">
         <v>22</v>
+      </c>
+      <c r="G56" s="2" t="s">
+        <v>688</v>
+      </c>
+      <c r="H56" s="2" t="s">
+        <v>689</v>
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.3">
@@ -3798,7 +4124,7 @@
         <v>663</v>
       </c>
     </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>268</v>
       </c>
@@ -3816,6 +4142,12 @@
       </c>
       <c r="F62" t="s">
         <v>17</v>
+      </c>
+      <c r="G62" s="2" t="s">
+        <v>680</v>
+      </c>
+      <c r="H62" s="2" t="s">
+        <v>681</v>
       </c>
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.3">
@@ -3878,7 +4210,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>282</v>
       </c>
@@ -3896,6 +4228,12 @@
       </c>
       <c r="F66" t="s">
         <v>11</v>
+      </c>
+      <c r="G66" s="2" t="s">
+        <v>700</v>
+      </c>
+      <c r="H66" s="2" t="s">
+        <v>701</v>
       </c>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.3">
@@ -3918,7 +4256,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>290</v>
       </c>
@@ -3936,6 +4274,12 @@
       </c>
       <c r="F68" t="s">
         <v>22</v>
+      </c>
+      <c r="G68" s="2" t="s">
+        <v>684</v>
+      </c>
+      <c r="H68" s="2" t="s">
+        <v>685</v>
       </c>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.3">
@@ -4144,7 +4488,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>339</v>
       </c>
@@ -4163,8 +4507,14 @@
       <c r="F79" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="G79" s="2" t="s">
+        <v>682</v>
+      </c>
+      <c r="H79" s="2" t="s">
+        <v>683</v>
+      </c>
+    </row>
+    <row r="80" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>344</v>
       </c>
@@ -4182,6 +4532,12 @@
       </c>
       <c r="F80" t="s">
         <v>22</v>
+      </c>
+      <c r="G80" s="2" t="s">
+        <v>708</v>
+      </c>
+      <c r="H80" s="2" t="s">
+        <v>709</v>
       </c>
     </row>
     <row r="81" spans="1:8" x14ac:dyDescent="0.3">
@@ -4370,7 +4726,7 @@
         <v>669</v>
       </c>
     </row>
-    <row r="90" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>382</v>
       </c>
@@ -4388,6 +4744,12 @@
       </c>
       <c r="F90" t="s">
         <v>17</v>
+      </c>
+      <c r="G90" s="2" t="s">
+        <v>690</v>
+      </c>
+      <c r="H90" s="2" t="s">
+        <v>691</v>
       </c>
     </row>
     <row r="91" spans="1:8" x14ac:dyDescent="0.3">
@@ -4470,7 +4832,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="95" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>399</v>
       </c>
@@ -4488,6 +4850,12 @@
       </c>
       <c r="F95" t="s">
         <v>11</v>
+      </c>
+      <c r="G95" s="2" t="s">
+        <v>694</v>
+      </c>
+      <c r="H95" s="2" t="s">
+        <v>695</v>
       </c>
     </row>
     <row r="96" spans="1:8" x14ac:dyDescent="0.3">
@@ -4510,7 +4878,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>409</v>
       </c>
@@ -4530,7 +4898,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>414</v>
       </c>
@@ -4550,7 +4918,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>416</v>
       </c>
@@ -4569,8 +4937,14 @@
       <c r="F99" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G99" s="2" t="s">
+        <v>702</v>
+      </c>
+      <c r="H99" s="2" t="s">
+        <v>703</v>
+      </c>
+    </row>
+    <row r="100" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>419</v>
       </c>
@@ -4590,7 +4964,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>424</v>
       </c>
@@ -4610,7 +4984,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>428</v>
       </c>
@@ -4630,7 +5004,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>433</v>
       </c>
@@ -4650,7 +5024,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>438</v>
       </c>
@@ -4669,8 +5043,14 @@
       <c r="F104" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G104" s="2" t="s">
+        <v>692</v>
+      </c>
+      <c r="H104" s="2" t="s">
+        <v>693</v>
+      </c>
+    </row>
+    <row r="105" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>443</v>
       </c>
@@ -4689,8 +5069,14 @@
       <c r="F105" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G105" s="2" t="s">
+        <v>710</v>
+      </c>
+      <c r="H105" s="2" t="s">
+        <v>711</v>
+      </c>
+    </row>
+    <row r="106" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>446</v>
       </c>
@@ -4710,7 +5096,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>451</v>
       </c>
@@ -4730,7 +5116,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>454</v>
       </c>
@@ -4750,7 +5136,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>459</v>
       </c>
@@ -4770,7 +5156,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>463</v>
       </c>
@@ -4790,7 +5176,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>468</v>
       </c>
@@ -4810,7 +5196,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>471</v>
       </c>
@@ -4830,7 +5216,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>472</v>
       </c>
@@ -4849,8 +5235,14 @@
       <c r="F113" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G113" s="2" t="s">
+        <v>686</v>
+      </c>
+      <c r="H113" s="2" t="s">
+        <v>687</v>
+      </c>
+    </row>
+    <row r="114" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>477</v>
       </c>
@@ -4870,7 +5262,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>482</v>
       </c>
@@ -4890,7 +5282,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>486</v>
       </c>
@@ -4910,7 +5302,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>488</v>
       </c>
@@ -4930,7 +5322,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>493</v>
       </c>
@@ -4950,7 +5342,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>498</v>
       </c>
@@ -4970,7 +5362,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>499</v>
       </c>
@@ -4990,7 +5382,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>504</v>
       </c>
@@ -5010,7 +5402,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>509</v>
       </c>
@@ -5029,8 +5421,14 @@
       <c r="F122" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G122" s="2" t="s">
+        <v>704</v>
+      </c>
+      <c r="H122" s="2" t="s">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="123" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>514</v>
       </c>
@@ -5050,7 +5448,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>515</v>
       </c>
@@ -5070,7 +5468,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>520</v>
       </c>
@@ -5090,7 +5488,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>524</v>
       </c>
@@ -5110,7 +5508,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
         <v>528</v>
       </c>
@@ -5130,7 +5528,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
         <v>531</v>
       </c>

</xml_diff>

<commit_message>
docs: update related answer quiz 4
</commit_message>
<xml_diff>
--- a/raw_csv_quiz/Quiz_Week04.xlsx
+++ b/raw_csv_quiz/Quiz_Week04.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\LearningHub\ai-2y-journey\06-other\flashcard-app\raw_csv_quiz\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CE04C0E-3896-4444-963E-C6BC15CB9DF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{082AE168-3A82-48AC-9FC8-71ED1EF34BDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2988" yWindow="792" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Questions" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1098" uniqueCount="712">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1132" uniqueCount="746">
   <si>
     <t>Question</t>
   </si>
@@ -2475,6 +2475,346 @@
 IAM Access Advisor (Option A): The Room Logs. It shows that "User A" entered the Breakroom and the Server Room, but not the Executive Suite.
 IAM Credentials Report (The Answer): The Manager's Spreadsheet. It lists every employee and exactly when their keycard was last scanned at the front gate. If the spreadsheet says "Last Scanned: January" and it's now April, you know it's time to deactivate that card. (This Answer)
 Key Exam Keyword: Whenever you need to audit or get a list/report of all users and their credential age/last used date, the answer is IAM Credentials Report.</t>
+  </si>
+  <si>
+    <t>C. Compute Savings Plans.
+Why is this the answer?
+Compute Savings Plans are the most flexible "commitment-based" pricing model AWS offers. They were specifically designed to solve the rigidity issues of older models.
+Massive Flexibility: Unlike other plans, these apply to your usage regardless of the service. If you move your code from an EC2 instance to a Lambda function or a Fargate container, the discount automatically follows you.
+No Geographic or Hardware Ties: They apply regardless of the Region (e.g., US-East-1 vs. Tokyo), Instance Family (e.g., moving from a t3 to an m5), or Operating System.
+Automatic Application: You simply commit to a consistent amount of spend (e.g., $10/hour for 1 or 3 years), and AWS automatically applies the discount to the highest-priced eligible usage first.
+Deep Savings: You can save up to 66% compared to On-Demand prices while maintaining the freedom to change your architecture.
+Why the other options are wrong:
+A. Standard Reserved Instances: These are the most "rigid." You are locked into a specific instance family, size, and region. They do not cover Lambda or Fargate.
+B. EC2 Instance Savings Plans: While these are a "Savings Plan," they are less flexible than the Compute version. They lock you into a specific instance family in a specific region (e.g., M5 instances in N. Virginia). They offer higher discounts (up to 72%) but much less freedom.
+D. Convertible Reserved Instances: These allow you to manually "exchange" your reservation for a different type, but it is a manual process and they do not cover Lambda or Fargate.</t>
+  </si>
+  <si>
+    <t>Think of your AWS commitment like a Gift Card:
+Standard Reserved Instance (Option A): This is a voucher for a Specific Item (e.g., "One specific Blue Shirt, Size Medium, at the New York store"). If you grow out of the shirt or want a red one, you're out of luck.
+EC2 Instance Savings Plan (Option B): This is a gift card for One Brand (e.g., "Any shirt from the Nike section in New York").
+Compute Savings Plans (The Answer): This is a General Mall Gift Card. You can buy a shirt (EC2), a pair of shoes (Fargate), or a hat (Lambda) at any store in the mall, in any city. (This Answer)
+Key Exam Keyword: Whenever you see "EC2, Lambda, and Fargate" mentioned together for a discount, the answer is always Compute Savings Plans.</t>
+  </si>
+  <si>
+    <t>D. CPU clock speed.
+Why is this the answer?
+When we talk about storage (specifically Amazon S3), the costs are determined by how you store and access your data, not the performance of the processor on the server.
+Storage Class Tiers (Option A): This is a major driver. Storing data in S3 Standard is more expensive than S3 Glacier. You pay for the "durability and availability" level you choose.
+PUT/GET Request Volume (Option B): You are charged for "actions" taken on your data. Every time you upload a file (PUT) or download/read a file (GET), it costs a tiny fraction of a cent. High-frequency applications will see this as a significant cost driver.
+Lifecycle Transitions (Option C): There is a cost associated with moving data between tiers (e.g., moving an object from S3 Standard to S3 Glacier using a Lifecycle Policy).
+CPU Clock Speed: This is a Compute metric, not a storage metric. You pay for CPU performance when renting EC2 instances, but S3 storage costs are independent of the hardware's clock speed.
+Why the other options are wrong:
+A, B, and C are all standard pillars of the S3 pricing model. Along with Data Transfer Out (moving data from S3 to the internet), these form the core "drivers" that determine your monthly storage bill.</t>
+  </si>
+  <si>
+    <t>Think of AWS Storage like renting a Physical Self-Storage Unit:
+Storage Class (A): Do you want a climate-controlled unit (Standard) or a dusty basement (Glacier)?
+Requests (B): Every time you open the lock to put something in or take something out, the facility charges a small "access fee."
+Lifecycle Transitions (C): The fee the facility charges to move your boxes from the expensive front room to the cheaper back warehouse.
+CPU Clock Speed (The Answer): This would be like the facility charging you based on how fast the truck's engine was that delivered your boxes. It doesn't matter to the storage company; they only care about the space you use and how often you visit. (This Answer)
+Key Exam Keyword: When looking for Storage Costs, look for Gigabytes (GB), Requests, Data Transfer, and Storage Class. Ignore anything related to CPU or RAM.</t>
+  </si>
+  <si>
+    <t>B. AWS Key Management Service (KMS).
+Why is this the answer?
+AWS KMS is the core service for managing cryptographic keys across the AWS ecosystem. When a company needs "full control," they specifically use Customer Managed Keys (CMKs).
+Customer Managed Keys (CMKs): Unlike "AWS Managed Keys" (which AWS creates and rotates for you), Customer Managed Keys are created by you. You control the key policies (who can use them) and their lifecycle.
+Rotation Control: With CMKs, you have two ways to handle rotation:Automatic Rotation: You can flip a switch and have AWS rotate the key material for you every year (or a custom frequency between 90 days and 7 years).Manual Rotation: You can choose to create a new key and update your application or S3 bucket to use that new key at any time.
+S3 Integration: S3 integrates seamlessly with KMS for Server-Side Encryption (SSE-KMS). You simply provide the KMS Key ID to the bucket, and S3 handles the heavy lifting of encrypting every object you upload.Auditing: Because you own the key, every time it is used to encrypt or decrypt data, a log is sent to AWS CloudTrail, giving you a complete audit trail of your data access.
+Why the other options are wrong:
+A. AWS Certificate Manager (ACM): This manages SSL/TLS certificates for websites (data in transit). It is not used for encrypting files sitting in a storage bucket (data at rest).
+C. Amazon Inspector: This is a vulnerability scanner. It checks your servers for security "holes" or unpatched software, but it doesn't manage encryption keys.
+D. AWS Shield: This is a DDoS protection service. It stops hackers from flooding your website with traffic to crash it; it has nothing to do with S3 encryption.</t>
+  </si>
+  <si>
+    <t>Think of your S3 data like your Valuables in a Safe:
+AWS Managed Key: This is like a safe provided by a hotel. They have a spare key, and they change the locks on their own schedule. You're safe, but you don't have total control.
+Customer Managed Key (KMS - The Answer): This is your Personal Safe. You bought the lock, you have the only keys, and you decide exactly when to change the combination or who is allowed to touch it. (This Answer)
+Key Exam Keyword: Whenever you see "Key rotation," "Full control over keys," or "Encryption at rest," the answer is AWS KMS.</t>
+  </si>
+  <si>
+    <t>C. AWS WAF with a Web ACL attached to the ALB.
+Why is this the answer?
+AWS WAF (Web Application Firewall) is designed specifically to protect web applications by inspecting the content of HTTP and HTTPS requests.
+Layer 7 Visibility: Unlike standard firewalls that only see IP addresses and ports, AWS WAF operates at the Application Layer (Layer 7). It can "read" the query strings, headers, and request bodies where SQL injection payloads are hidden.
+Web ACLs and Rules: You create a Web Access Control List (Web ACL) and add rules specifically designed to detect SQL injection patterns. AWS even provides Managed Rule Groups that are pre-configured to block these common attacks, so you don't have to write the regex yourself.
+ALB Integration: AWS WAF integrates natively with the Application Load Balancer. Once you attach the Web ACL to the ALB, every incoming request is inspected and blocked before it ever reaches your web servers.
+Real-Time Blocking: Because it sits "inline," it can drop malicious requests in real-time, preventing the SQL command from ever reaching your database.
+Why the other options are wrong:
+A. AWS Shield Standard: This provides automatic protection against Layer 3 and 4 DDoS attacks (like SYN floods). It does not inspect the "application payload" and therefore cannot stop a SQL injection.
+B. AWS Network Firewall: This is a VPC-level firewall for Layer 3 through Layer 7. While powerful, it is typically used for inspecting all traffic across the network (like filtering outbound domains). For a specific web app behind an ALB, AWS WAF is the purpose-built, more cost-effective choice for SQLi/XSS.
+D. Amazon GuardDuty: This is a threat detection service that looks at logs to find "after-the-fact" evidence of a compromise. It is not an "inline" tool and cannot block a specific HTTP request as it happens.</t>
+  </si>
+  <si>
+    <t>Think of your web application as an Office Building and the ALB as the Front Desk:
+AWS Shield (Option A): Like a gate that stops a massive crowd from blocking the street so no one can get to the building (DDoS).
+Network Firewall (Option B): Like a security checkpoint at the parking lot entrance that checks if the cars are allowed on the property.
+AWS WAF (The Answer): Like a Mailroom Inspector who opens every envelope sent to the building. If they find a "threat" written inside the letter (like a malicious SQL command), they shred the letter immediately so the employees inside never see it. (This Answer)
+Key Exam Keyword: Whenever you see "SQL Injection," "Cross-Site Scripting (XSS)," or "Application Layer (Layer 7) attacks," the answer is almost always AWS WAF.</t>
+  </si>
+  <si>
+    <t>C. Reserved Instances (or B. Savings Plans—both are correct for "long-term stable," but C is the traditional answer for this specific exam phrasing).
+Why is this the answer?
+For a "stable" workload—meaning your servers are running 24/7 and you don't plan on turning them off for at least a year—you want to move away from the expensive "pay-as-you-go" model.
+Commitment for Discount: Both Reserved Instances (RIs) and Savings Plans require a commitment of 1 or 3 years. In exchange for this "guaranteed" business, AWS gives you a massive discount (up to 72%).
+Steady State: Because the workload is "stable," you aren't worried about being locked into a contract. You know you'll need the capacity, so paying a lower rate for that certainty is the most cost-effective move.
+Capacity Reservation: While Savings Plans are more flexible, Standard Reserved Instances can also provide a "capacity reservation," ensuring that the specific server type you need is always available in a specific Availability Zone.
+Why the other options are wrong:
+A. On-Demand: This is for short-term, unpredictable workloads. It is the most expensive model because you are paying for the flexibility to turn the server off at any second.
+D. Spot Instances: These are for interruptible workloads. While they are the cheapest (90% off), they are terrible for a "stable" workload because AWS can take the server away with only a 2-minute notice.</t>
+  </si>
+  <si>
+    <t>Think of these pricing models like your Living Situation:
+On-Demand (Option A): Staying in a Hotel. It’s expensive per night, but you can leave whenever you want. Great for a 2-day trip (short-term).
+Spot Instances (Option D): Couch Surfing. It’s almost free, but the owner can kick you out the moment their cousin comes to visit. You can't rely on it for a "stable" life.
+Reserved Instances / Savings Plans (The Answer): Signing a 1-Year Lease on an apartment. You commit to staying for a year, and in return, the monthly rent is much lower than a hotel. (This Answer)
+Key Exam Keyword: Whenever you see "Stable," "Predictable," or "Long-term," look for Reserved Instances or Savings Plans.</t>
+  </si>
+  <si>
+    <t>C. Inbound data transfer (data into AWS) is generally free, while outbound data transfer (data out to the internet) is charged.
+Why is this the answer?
+AWS follows a "Data Gravity" strategy. They make it easy and free to get your data into their ecosystem, but charge you when that data leaves.
+Inbound (Ingress) = $0.00: AWS generally does not charge you for data coming into their network from the internet. Whether you are uploading a 10TB dataset to S3 or sending millions of API requests to an EC2 instance, the "Data Transfer In" line item on your bill will almost always be zero.
+Outbound (Egress) = Tiered Pricing: Data leaving AWS to go to the internet is where the costs accumulate.
+The First 100 GB/month: This is free under the AWS Free Tier (which applies to both new and existing accounts).
+Beyond 100 GB: You are charged per GB based on a tiered structure. In many regions, the next 10 TB starts at approximately $0.09 per GB. The more you transfer, the lower the price per GB becomes.
+The "Middle" Costs: While not in the primary question, it's important to remember that data moving between AWS Regions (Inter-Region) or between Availability Zones (Inter-AZ) also carries a cost (typically $0.01 to $0.02 per GB).
+Why the other options are wrong:
+A. Both are free: If this were true, companies like Netflix would have much smaller AWS bills! Outbound data transfer is actually one of the largest cost drivers for high-traffic applications.
+B. Both charged at same rate: This is incorrect because of the strategic "free inbound" rule. AWS wants to lower the barrier for you to move your workloads to their cloud.
+D. Outbound free / Inbound charged: This is the opposite of how AWS (and most major cloud providers) operates. Charging for inbound data would discourage customers from migrating their data to AWS.</t>
+  </si>
+  <si>
+    <t>Think of AWS data transfer like the Water Pipes in your house:
+Inbound (The Answer): This is like the Rain falling into a collection barrel you've set up. The clouds (the internet) don't charge you to let the water fall into your barrel (AWS). (This Answer)
+Outbound: This is like Turning on the Tap. The water company (AWS) charges you for every gallon that leaves the pipes to go down the drain or water your lawn.
+Key Exam Keyword: Whenever you see "Data Transfer In," think Free. Whenever you see "Data Transfer Out (to Internet)," think Tiered Charges.</t>
+  </si>
+  <si>
+    <t>A. Middle-man Managed Keys.
+Why is this the answer?
+AWS Key Management Service (KMS) uses a very specific hierarchy of keys to manage security. "Middle-man Managed Keys" is a made-up term and does not exist in the AWS ecosystem.
+The three legitimate types of KMS keys are:
+AWS Owned Keys (C): These are keys that AWS services (like DynamoDB or S3) own and use in multiple AWS accounts. You cannot view, manage, or audit these keys. They are used to provide basic encryption for services at no cost to you.
+AWS Managed Keys (B): These are created in your account automatically when you use a service that integrates with KMS. You can see them in your KMS console (they usually have an alias like aws/s3), but you cannot delete or change their policies. AWS handles the rotation for you.
+Customer Managed Keys (D): These are keys you create. You have full control over them, including defining who can use them (Key Policies), enabling/disabling them, and setting up manual or automatic rotation. These are the keys you use when you have strict compliance requirements.
+Why the other options are wrong:
+B, C, and D are the three actual pillars of the KMS service. Any question asking you to identify a "KMS Key Type" will involve these three categories.</t>
+  </si>
+  <si>
+    <t>The correct answer is A. Middle-man Managed Keys.
+Why is this the answer?
+AWS Key Management Service (KMS) uses a very specific hierarchy of keys to manage security. "Middle-man Managed Keys" is a made-up term and does not exist in the AWS ecosystem.
+The three legitimate types of KMS keys are:
+AWS Owned Keys (C): These are keys that AWS services (like DynamoDB or S3) own and use in multiple AWS accounts. You cannot view, manage, or audit these keys. They are used to provide basic encryption for services at no cost to you.
+AWS Managed Keys (B): These are created in your account automatically when you use a service that integrates with KMS. You can see them in your KMS console (they usually have an alias like aws/s3), but you cannot delete or change their policies. AWS handles the rotation for you.
+Customer Managed Keys (D): These are keys you create. You have full control over them, including defining who can use them (Key Policies), enabling/disabling them, and setting up manual or automatic rotation. These are the keys you use when you have strict compliance requirements.
+Why the other options are wrong:
+B, C, and D are the three actual pillars of the KMS service. Any question asking you to identify a "KMS Key Type" will involve these three categories.
+📝 Newbie Note: The "Hotel Safe" Analogy
+To remember the difference between the three real keys, think of a hotel stay:
+AWS Owned: The Hotel's Main Vault. You know it exists, and the hotel uses it to protect things in the building, but you never see it and don't have a key to it.
+AWS Managed: The Safe in your Room. The hotel put it there for you. You can use it, but you didn't choose the model, and the manager has a master code to help if you're locked out.
+Customer Managed: Your Own Padlock. You brought it from home, you set the combination, and you are the only one who can open it. If you lose the code, the hotel can't help you. (This Answer)
+Key Exam Keyword: There are only three types of KMS keys. If you see anything that sounds like "Third-party," "Middle-man," or "Global Managed," it is a distractor.</t>
+  </si>
+  <si>
+    <t>C. Accessing AWS services in the same Region via an Internet Gateway (specifically referring to data transfer inbound to AWS).
+Note: There is a slight nuance in this question. While the Internet Gateway itself is free, the specific reason for "no charge" in this context is that AWS does not charge for Inbound Data Transfer from the internet.
+Why is this the answer?
+AWS pricing is designed to encourage you to bring data into their ecosystem.
+Inbound is Free: Data coming from the internet through an Internet Gateway into an AWS service (like an EC2 instance or an S3 bucket) in the same region is generally free of charge.
+Service Specifics: Accessing "Public" AWS services (like S3 or DynamoDB) from within the same region typically incurs no data transfer charges, provided you aren't crossing Availability Zone boundaries in a way that triggers "Inter-AZ" fees.
+Why the other options are wrong:
+A. Between different AWS Regions: This is called Inter-Region Data Transfer. This is almost always charged (e.g., $0.01 or $0.02 per GB) because AWS has to use its global backbone network to move that data across the world.
+B. Across two different Availability Zones: This is Inter-AZ Data Transfer. Even within the same region, moving data between AZs usually costs $0.01 per GB for both the "sending" and "receiving" components.
+D. Using a NAT Gateway: This is a common "cost trap." NAT Gateways have two costs: an hourly usage fee and a data processing charge (approx. $0.045 per GB). Even if the data is going to a free destination, the "processing" through the gateway is not free.</t>
+  </si>
+  <si>
+    <t>Think of your AWS Region like a Shopping Mall:
+Internet Gateway (The Answer): This is the Main Entrance. The mall doesn't charge you to walk through the front door and bring your bags (data) inside. (This Answer)
+Between Regions (Option A): This is like taking a shuttle bus from a mall in New York to a mall in Los Angeles. You definitely have to pay for that ticket.
+Between Availability Zones (Option B): This is like moving your bags from one wing of the mall to another via a private courier. There is a small "convenience fee" for moving between the different buildings.
+NAT Gateway (Option D): This is like using a Private Valet to carry your bags. Even if the entrance is free, you have to pay the valet for the "work" they do carrying the bags.
+Key Exam Keyword: Whenever you see "Inbound" or "Same Region / Same AZ," look for No Charge. Whenever you see "Inter-Region," "Inter-AZ," or "NAT Gateway," expect a Fee.</t>
+  </si>
+  <si>
+    <t>D. There is no automatic rotation; it must be done manually.
+Why is this the answer?
+This is a very specific technical detail that often appears on AWS security and practitioner exams. It centers on the "Origin" of the key material.
+Origin of the Key: When you create a KMS key, the default origin is AWS_KMS, where AWS generates the random numbers for you. For these keys, AWS can easily generate new numbers (rotate) every year.
+External Origin (BYOK): When you import your own key material (Bring Your Own Key), the origin is set to EXTERNAL.
+The Responsibility Shift: Because the key material came from your infrastructure (not AWS), AWS does not have the authority or the ability to "generate" a new version of your external secret. Therefore, the Enable Automatic Rotation checkbox is literally grayed out or unavailable for these keys.
+How to Rotate: To rotate an imported key, you must:
+Create a new KMS key.
+Import new key material into that new key.
+Update your application (or a Key Alias) to point to the new Key ID.
+Why the other options are wrong:
+A &amp; B: Automatic rotation (whether 365 or 90 days) is only supported for symmetric keys where AWS generated the material.
+C: AWS Support does not have access to your keys and cannot perform cryptographic operations or rotations for you. One of the main selling points of KMS is that even AWS employees cannot see your unencrypted keys.</t>
+  </si>
+  <si>
+    <t>Think of your KMS key as a Security Gate:
+AWS Generated Key: This is like a gate provided by the manufacturer that comes with an automatic code-changer. Every year, the manufacturer's system automatically updates the code for you.
+Imported Key Material (The Answer): This is a gate where you provided the lock. Because it’s your specific lock from your own locksmith, the gate manufacturer doesn't have the "master code" or the right to change it. If you want a new code, you have to go get a new lock yourself and swap it out. (This Answer)
+Key Exam Keyword: If a question mentions "Imported Key Material" or "EXTERNAL Origin," automatic rotation is NOT an option. You must do it manually by creating a new key.</t>
+  </si>
+  <si>
+    <t>C. Place AWS Global Accelerator in front of the ALB.
+Why is this the answer?
+This is a common "Design Pattern" question that tests your ability to combine services to meet specific networking and security requirements.
+The ALB Limitation: An Application Load Balancer (ALB) is the only load balancer that natively supports AWS WAF (Layer 7 protection). However, ALBs use hostnames (DNS) and their underlying IP addresses can change frequently.
+The Global Accelerator Solution: AWS Global Accelerator provides you with two static Anycast IP addresses. These IPs do not change.
+The Integration: You point the Global Accelerator to your ALB as an "endpoint."
+External Users: See and whitelist the Static IPs of the Global Accelerator.
+Security: The AWS WAF remains attached to the ALB, inspecting the traffic as it passes through.
+Performance Bonus: Besides providing static IPs, Global Accelerator routes traffic over the AWS global network instead of the public internet, reducing latency and jitter for your users.
+Why the other options are wrong:
+A. WAF directly to an NLB: This is technically impossible. AWS WAF cannot be attached to a Network Load Balancer. NLBs operate at Layer 4 (TCP/UDP), while WAF needs to see Layer 7 (HTTP) to work.
+B. Elastic IP to WAF: You cannot attach an Elastic IP to a WAF Web ACL. WAF is a managed service "layer," not a network interface with an IP address.
+D. Route 53 to generate a static IP: Route 53 is a DNS service. While it can map names to IPs, it cannot "generate" or "create" a static IP for a service that doesn't natively support one.</t>
+  </si>
+  <si>
+    <t>Think of your web application like a Business:
+The ALB (The Business): It moves around to different offices. Every time it moves, its phone number (IP address) changes. Customers find it hard to keep track.
+AWS WAF (The Security Guard): The guard stands at the office door. He only works at this specific type of office (ALB).
+AWS Global Accelerator (The Answer): This is like a 1-800 Permanent Number. No matter which office the business moves to, the 1-800 number stays the same. Customers just call the 1-800 number, and it forwards the call to the current office where the Security Guard (WAF) is waiting. (This Answer)
+Key Exam Keyword: Whenever you see a requirement for "Static IP" combined with an "ALB" or "WAF," the answer is almost always Global Accelerator.</t>
+  </si>
+  <si>
+    <t>D. AWS Firewall Manager.
+Why is this the answer?
+AWS Firewall Manager is the "master controller" designed specifically for large organizations that need to maintain a consistent security posture across multiple AWS accounts.
+AWS Organizations Integration: It works directly with AWS Organizations. You designate an administrator account that can push security policies (like WAF rules or Shield Advanced protections) to every member account in the organization.
+"Set it and Forget it": You define your security policy once. Firewall Manager automatically applies that policy to existing resources and, more importantly, to newly created resources. If a developer in another account spins up a new Load Balancer, Firewall Manager will see it and automatically attach the mandatory WAF rules.
+Cross-Account Enforcement: If a user in a member account tries to delete or change a rule that was pushed by the Firewall Manager, the service will detect the change and automatically "revert" it to stay in compliance.
+Centralized Shield Advanced: It simplifies the deployment of Shield Advanced. Instead of manually enabling protection for every Elastic IP or CloudFront distribution in 50 different accounts, you can do it from one central dashboard.
+Why the other options are wrong:
+A. Amazon Macie: This is for data privacy and discovery. It scans S3 buckets for sensitive info like credit card numbers. It has nothing to do with WAF or Shield.
+B. AWS Config: While Firewall Manager uses AWS Config in the background to detect new resources, AWS Config itself is a compliance and auditing tool. It can tell you if a resource is "non-compliant," but it isn't the primary tool used to "centrally define and enforce" WAF rules across accounts.
+C. AWS GuardDuty: This is a threat detection service (the "Security Guard"). It watches logs for hackers but doesn't manage or deploy firewall rules.</t>
+  </si>
+  <si>
+    <t>Think of your AWS Organization like a Pizza Chain (like Domino's):
+Individual Accounts: These are the local pizza shops. Each shop has its own manager and staff.
+AWS WAF &amp; Shield: These are the Security Alarms and Health Rules for each shop.
+AWS Firewall Manager (The Answer): This is the Corporate Headquarters. Instead of hoping every local manager remembers to set the alarm correctly, Headquarters uses a central system to "push" the exact same security settings and recipes to every shop in the country. If a new shop opens tomorrow, the system automatically installs the alarms. (This Answer)
+Key Exam Keyword: Whenever you see "Centrally manage," "Across multiple accounts," or "Enforce WAF/Shield rules at scale," the answer is AWS Firewall Manager.</t>
+  </si>
+  <si>
+    <t>A. AWS Pricing Calculator.
+Why is this the answer?
+The AWS Pricing Calculator is a web-based planning tool that allows you to create an estimate for your AWS use cases before you actually commit to any spending or launch any instances.
+Modeling Architectures: You can add specific services (like an EC2 instance with a certain amount of RAM, or an S3 bucket with 500GB of storage) and see how the configuration affects the price.
+Pre-Provisioning: It is used during the design phase. You don't need an active AWS account or any running resources to use it.
+Transparent Estimates: It breaks down the costs into monthly and yearly totals, including upfront costs for things like Reserved Instances.
+Shareable Results: You can save your estimate and share the link with your manager or finance team to get budget approval before building the project.
+Why the other options are wrong:
+B. AWS Trusted Advisor: This tool looks at existing resources in your account and gives you recommendations on how to improve security, performance, and cost-efficiency (e.g., "You have an idle Load Balancer you should delete").
+C. AWS Cost Explorer: This is used to analyze past spending. It provides graphs and tables showing where your money went over the last 12–13 months and helps you forecast future spending based on that history.
+D. AWS Budgets: This is a tracking and alerting tool. You set a limit (e.g., "I don't want to spend more than $50/month"), and it sends you an email or SNS notification if your actual or forecasted costs exceed that limit.</t>
+  </si>
+  <si>
+    <t>Think of your AWS project like building a New House:
+AWS Pricing Calculator (The Answer): This is the Blueprint and Quote. You sit down with an architect before buying any wood to figure out how much the house will cost based on the number of rooms and the materials you choose. (This Answer)
+AWS Budgets (Option D): This is the Bank Alert on your phone that pings you when you've spent 80% of your construction loan.
+AWS Cost Explorer (Option C): This is your Credit Card Statement showing exactly how much you spent on wood and nails last month.
+AWS Trusted Advisor (Option B): This is the Home Inspector who walks through your already built house and tells you that you're wasting money by leaving the lights on in the basement.
+Key Exam Keyword: Whenever the question mentions "Estimating," "Before provisioning," or "Planning a use case," the answer is AWS Pricing Calculator.</t>
+  </si>
+  <si>
+    <t>C. Data transfer from the Internet to AWS (Inbound Data Transfer).
+Why is this the answer?
+AWS follows a "Data Gravity" strategy. They make it easy and free to get your data into their ecosystem, but they generally charge you when that data leaves or moves between major infrastructure boundaries.
+Inbound (Ingress) is Free: Whether you are uploading a massive 1TB image dataset for your ML research or receiving millions of HTTP requests from users, AWS does not charge for the data coming into their network from the internet.
+Encouraging Migration: By keeping inbound transfer free, AWS lowers the barrier for companies to move their workloads and data into the cloud.
+Applies to Most Services: This "Free Inbound" rule applies to Amazon S3, Amazon EC2, Amazon RDS, and most other core services.
+Why the other options are wrong:
+A. Between two different Regions: This is Inter-Region Data Transfer. Because the data has to travel across the AWS global backbone (e.g., from US-East-1 to Singapore), there is a cost (typically around $0.02 per GB).
+B. From AWS to the Internet (Outbound): This is the most common cost driver. After the first 100GB (which is free per month), AWS charges a tiered rate (starting around $0.09 per GB) for data leaving their network.
+D. Between two different AZs: This is Inter-AZ Data Transfer. Even though it stays within the same region, moving data between physically separate data centers (AZs) usually costs $0.01 per GB in each direction.</t>
+  </si>
+  <si>
+    <t>Think of an AWS Region like a Giant Shopping Mall:
+Inbound (The Answer): You can walk into the mall with as many shopping bags as you want. The mall doesn't charge you a "door fee" to bring things inside. (This Answer)
+Outbound (Option B): If you buy something and want to take it out to your car, you have to pay a "delivery/exit fee."
+Inter-Region (Option A): This is like taking a shuttle bus to a completely different mall in another city. That bus ticket costs money.
+Inter-AZ (Option D): This is like moving your shopping bags from the North Wing of the mall to the South Wing. Even though you're in the same mall, you have to pay the internal courier a small tip to move your stuff across the bridge.
+Key Exam Keyword: Whenever you see "Data Transfer In," think $0. Whenever you see "Outbound," "Inter-Region," or "Inter-AZ," expect a Fee.</t>
+  </si>
+  <si>
+    <t>B. HNSW-PQ compression.
+Why is this the answer?
+In high-scale RAG (Retrieval-Augmented Generation) deployments, Product Quantization (PQ) is the "magic bullet" for cost reduction because it fundamentally changes how vectors are stored in memory.
+Massive Compression: Standard vectors are usually stored in FP32 (32-bit floats) or FP16. If you have a 1536-dimensional vector (like OpenAI's), that is a lot of data. PQ breaks these vectors into smaller sub-vectors and replaces them with short "codebook" indices. This can reduce the memory footprint by 80% to 90%.
+HNSW + PQ: While HNSW (Hierarchical Navigable Small World) provides the extreme speed needed for production, it is notorious for high memory usage because it stores both the vectors and a complex graph structure. By adding PQ, you keep the search speed but drastically lower the RAM requirements of the cluster.
+The $75k to $10k Logic: In a typical cloud-hosted vector database, your bill is tied directly to the RAM (Instance size) required to keep your index "hot." Cutting your memory footprint by 7x–8x allows you to downsize your clusters from massive, high-memory instances to much smaller ones, resulting in the ~86% savings described.
+Why the other options are wrong:
+A. HNSW-FP16: Moving from FP32 to FP16 only cuts your storage in half (50% reduction). It is a good start, but it cannot achieve the ~85% reduction ($75k to $10k) required by the prompt.
+C. S3 Glacier Lifecycle: This is a trap! S3 Glacier is for "cold" storage. If you move your vectors to Glacier, you cannot search them. RAG requires the vector index to be "active" (usually in RAM or on NVMe SSDs) to retrieve context for the LLM in real-time.
+D. Consolidating Clusters: While this reduces "overhead" (like paying for multiple master nodes), it doesn't change the underlying data volume. If you have 1TB of vectors, you still need 1TB of capacity, whether it's in one cluster or five.</t>
+  </si>
+  <si>
+    <t>Key Exam Keyword: Whenever you see a question about "Reducing vector storage costs by 80%+" or "Optimizing HNSW memory," the answer is Product Quantization (PQ).</t>
+  </si>
+  <si>
+    <t>C. AWS Certificate Manager (ACM).
+Why is this the answer?
+AWS Certificate Manager (ACM) is the purpose-built service for handling the lifecycle of SSL/TLS certificates. These certificates are the "digital IDs" required to enable HTTPS, which ensures that data moving between a user’s browser and your server is encrypted (encryption in transit).
+Provisioning: You can request a new public certificate directly from AWS (issued by Amazon’s own Certificate Authority) or import one you purchased from a third party.
+Deployment: ACM integrates natively with other AWS services. You can "attach" a certificate to an Application Load Balancer (ALB), Amazon CloudFront, or API Gateway with just a few clicks.
+Managed Renewal: This is ACM's biggest benefit. If you use an Amazon-issued certificate that is currently in use by an AWS service, ACM handles the renewal process automatically. You never have to worry about your website going down because of an expired certificate.
+Cost: Public SSL/TLS certificates requested through ACM are free to use with integrated AWS services.
+Why the other options are wrong:
+A. AWS KMS (Key Management Service): This is used for managing encryption keys (like the ones used to encrypt S3 buckets or EBS volumes). It handles "encryption at rest" rather than managing SSL certificates for web traffic.
+B. AWS Secrets Manager: This is designed for storing secrets like database passwords or API keys. While you could technically store certificate files here as text, Secrets Manager does not "provision" or "deploy" SSL certificates to load balancers.
+D. SSM Parameter Store: Similar to Secrets Manager, this is used for configuration data and passwords. It is a storage tool, not a certificate management and deployment service.</t>
+  </si>
+  <si>
+    <t>Think of your website as a traveler and an SSL certificate as their Passport:
+The Passport (SSL Certificate): It proves the traveler is who they say they are and allows them to pass through security (encryption).
+AWS Certificate Manager (The Answer): This is the Passport Office. They issue the passport to you, verify your identity (Domain Validation), and most importantly, they automatically send you a new one in the mail before the old one expires so you never get stuck at the border. (This Answer)
+Key Exam Keyword: Whenever you see "SSL/TLS," "HTTPS," or "Certificate renewal," the answer is ACM.</t>
+  </si>
+  <si>
+    <t>A. The unit cost decreases.
+Why is this the answer?
+The "Volume Discounts" principle is a core part of the AWS Pay-as-you-go pricing philosophy. It is designed to reward customers for scaling their operations on the AWS platform.
+Tiered Pricing: Many services, particularly Amazon S3 (storage) and Data Transfer Out, use a tiered pricing model. For example, the price per GB for the first 50 TB of storage is higher than the price per GB for the next 450 TB.
+Economies of Scale: As AWS grows and more customers use more resources, AWS's own operational costs decrease. They pass these "economies of scale" back to the user in the form of lower unit prices.
+Automatic Application: You don't usually have to ask for these discounts; they are applied automatically as your monthly usage crosses the different thresholds (tiers) defined in the service's pricing page.
+Incentive to Consolidate: This principle is why many companies use Consolidated Billing (via AWS Organizations). By combining the usage of 10 different accounts, they can reach the cheaper, higher-volume tiers much faster than they would individually.
+Why the other options are wrong:
+B. The unit cost increases: This would be a "scarcity" model. AWS is designed for infinite scale, so they want to encourage more usage, not penalize it.
+C. The unit cost remains unchanged: While some services have a "flat" rate (like certain Lambda executions), the primary principle AWS advertises regarding growth is the volume discount.
+D. Your resources will be limited: While there are "Service Quotas" to prevent accidental overspending, the pricing principle is about cost, not limits. AWS wants to provide as many resources as you are willing to pay for.</t>
+  </si>
+  <si>
+    <t>Think of AWS like a Big-Box Wholesale Club (like Costco or Sam's Club):
+On-Demand: Buying a single bottle of water at a convenience store is expensive.
+Volume Discount (The Answer): Buying a 24-pack of water at the warehouse. Because you are buying a large volume, the "price per bottle" (the unit cost) is significantly lower than if you bought them one by one. (This Answer)
+Key Exam Keyword: Whenever you see "Volume Discounts" or "Economies of Scale," the answer is always Lower unit cost as usage increases.</t>
+  </si>
+  <si>
+    <t>D. AWS Shield Advanced.
+Why is this the answer?
+While the company already has a Business Support plan, that plan alone does not grant access to the DDoS Response Team (DRT)—now often referred to as the Shield Response Team (SRT). Access to this specialized group of engineers is a specific benefit of the AWS Shield Advanced subscription.
+Specialized Support (SRT/DRT): Only Shield Advanced customers (who also have a Business or Enterprise support plan) can engage the SRT. These experts provide 24/7 assistance to help you triage, analyze, and mitigate complex Layer 3, 4, or 7 DDoS attacks.
+Proactive Engagement: With Shield Advanced, the SRT can proactively contact you if they detect an attack on your resources that is causing your Route 53 health checks to fail.
+Manual Mitigations: The SRT can help you write and apply custom AWS WAF rules on your behalf during an active incident to block sophisticated application-layer attacks.
+Requirement Pairing: To get SRT/DRT support, you must have both an AWS Shield Advanced subscription and a Business or Enterprise support plan. Since the company already has Business Support, they just need to add Shield Advanced.
+Why the other options are wrong:
+A. AWS Shield Standard: This is the free version enabled for everyone. It provides automatic protection against common network/transport layer attacks but does not provide access to the specialized response team or advanced metrics.
+B. AWS Enterprise Support: While this plan gives you a Technical Account Manager (TAM) and the highest level of general support, it does not "unlock" the DDoS Response Team unless you also subscribe to Shield Advanced.
+C. AWS WAF: This is the tool (the "firewall") used to block malicious web requests. While it is part of a DDoS strategy, simply having WAF does not give you access to the AWS human experts in the DRT.</t>
+  </si>
+  <si>
+    <t>Think of your AWS resources as a High-End Jewelry Store:
+Shield Standard (Option A): This is the Automated Alarm System. It's always on and stops basic burglars (simple attacks) automatically at no cost to you.
+AWS WAF (Option C): This is the Bulletproof Glass on the display cases. It's a tool you put in place to stop specific types of theft (web exploits).
+AWS Shield Advanced (The Answer): This is like having a Private Security Firm on retainer. Because you pay for the premium service, you get access to a Rapid Response SWAT Team (the DRT) that will rush to your store during a complex heist to personally fight off the attackers and help you fix the glass. (This Answer)
+Key Exam Keyword: Whenever a question asks about the "DDoS Response Team (DRT)" or "Shield Response Team (SRT)," the answer must include AWS Shield Advanced.</t>
   </si>
 </sst>
 </file>
@@ -2970,7 +3310,7 @@
         <v>671</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>32</v>
       </c>
@@ -2988,6 +3328,12 @@
       </c>
       <c r="F7" t="s">
         <v>22</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>722</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>723</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
@@ -3428,7 +3774,7 @@
         <v>707</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>134</v>
       </c>
@@ -3446,6 +3792,12 @@
       </c>
       <c r="F29" t="s">
         <v>17</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>714</v>
+      </c>
+      <c r="H29" s="2" t="s">
+        <v>715</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.3">
@@ -3508,7 +3860,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>151</v>
       </c>
@@ -3526,6 +3878,12 @@
       </c>
       <c r="F33" t="s">
         <v>22</v>
+      </c>
+      <c r="G33" s="2" t="s">
+        <v>736</v>
+      </c>
+      <c r="H33" s="2" t="s">
+        <v>737</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.3">
@@ -3568,7 +3926,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>165</v>
       </c>
@@ -3586,6 +3944,12 @@
       </c>
       <c r="F36" t="s">
         <v>11</v>
+      </c>
+      <c r="G36" s="2" t="s">
+        <v>716</v>
+      </c>
+      <c r="H36" s="2" t="s">
+        <v>717</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.3">
@@ -3926,7 +4290,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>232</v>
       </c>
@@ -3944,6 +4308,12 @@
       </c>
       <c r="F53" t="s">
         <v>47</v>
+      </c>
+      <c r="G53" s="2" t="s">
+        <v>742</v>
+      </c>
+      <c r="H53" s="2" t="s">
+        <v>743</v>
       </c>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.3">
@@ -4190,7 +4560,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>281</v>
       </c>
@@ -4208,6 +4578,12 @@
       </c>
       <c r="F65" t="s">
         <v>22</v>
+      </c>
+      <c r="G65" s="2" t="s">
+        <v>720</v>
+      </c>
+      <c r="H65" s="2" t="s">
+        <v>721</v>
       </c>
     </row>
     <row r="66" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
@@ -4322,7 +4698,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>302</v>
       </c>
@@ -4340,6 +4716,12 @@
       </c>
       <c r="F71" t="s">
         <v>17</v>
+      </c>
+      <c r="G71" s="2" t="s">
+        <v>732</v>
+      </c>
+      <c r="H71" s="2" t="s">
+        <v>733</v>
       </c>
     </row>
     <row r="72" spans="1:8" x14ac:dyDescent="0.3">
@@ -4772,7 +5154,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="92" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>388</v>
       </c>
@@ -4790,6 +5172,12 @@
       </c>
       <c r="F92" t="s">
         <v>47</v>
+      </c>
+      <c r="G92" s="2" t="s">
+        <v>724</v>
+      </c>
+      <c r="H92" s="2" t="s">
+        <v>725</v>
       </c>
     </row>
     <row r="93" spans="1:8" x14ac:dyDescent="0.3">
@@ -4812,7 +5200,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="94" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>394</v>
       </c>
@@ -4830,6 +5218,12 @@
       </c>
       <c r="F94" t="s">
         <v>22</v>
+      </c>
+      <c r="G94" s="2" t="s">
+        <v>712</v>
+      </c>
+      <c r="H94" s="2" t="s">
+        <v>713</v>
       </c>
     </row>
     <row r="95" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
@@ -4944,7 +5338,7 @@
         <v>703</v>
       </c>
     </row>
-    <row r="100" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>419</v>
       </c>
@@ -4962,6 +5356,12 @@
       </c>
       <c r="F100" t="s">
         <v>11</v>
+      </c>
+      <c r="G100" s="2" t="s">
+        <v>738</v>
+      </c>
+      <c r="H100" t="s">
+        <v>739</v>
       </c>
     </row>
     <row r="101" spans="1:8" x14ac:dyDescent="0.3">
@@ -5136,7 +5536,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="109" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>459</v>
       </c>
@@ -5154,6 +5554,12 @@
       </c>
       <c r="F109" t="s">
         <v>22</v>
+      </c>
+      <c r="G109" s="2" t="s">
+        <v>718</v>
+      </c>
+      <c r="H109" s="2" t="s">
+        <v>719</v>
       </c>
     </row>
     <row r="110" spans="1:8" x14ac:dyDescent="0.3">
@@ -5382,7 +5788,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="121" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>504</v>
       </c>
@@ -5400,6 +5806,12 @@
       </c>
       <c r="F121" t="s">
         <v>22</v>
+      </c>
+      <c r="G121" s="2" t="s">
+        <v>726</v>
+      </c>
+      <c r="H121" s="2" t="s">
+        <v>727</v>
       </c>
     </row>
     <row r="122" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
@@ -5428,7 +5840,7 @@
         <v>705</v>
       </c>
     </row>
-    <row r="123" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>514</v>
       </c>
@@ -5446,6 +5858,12 @@
       </c>
       <c r="F123" t="s">
         <v>47</v>
+      </c>
+      <c r="G123" s="2" t="s">
+        <v>734</v>
+      </c>
+      <c r="H123" s="2" t="s">
+        <v>735</v>
       </c>
     </row>
     <row r="124" spans="1:8" x14ac:dyDescent="0.3">
@@ -5548,7 +5966,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
         <v>535</v>
       </c>
@@ -5568,7 +5986,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
         <v>538</v>
       </c>
@@ -5588,7 +6006,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
         <v>541</v>
       </c>
@@ -5608,7 +6026,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
         <v>542</v>
       </c>
@@ -5628,7 +6046,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
         <v>543</v>
       </c>
@@ -5648,7 +6066,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
         <v>548</v>
       </c>
@@ -5667,8 +6085,14 @@
       <c r="F134" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G134" s="2" t="s">
+        <v>728</v>
+      </c>
+      <c r="H134" s="2" t="s">
+        <v>729</v>
+      </c>
+    </row>
+    <row r="135" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
         <v>553</v>
       </c>
@@ -5688,7 +6112,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
         <v>556</v>
       </c>
@@ -5708,7 +6132,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
         <v>561</v>
       </c>
@@ -5727,8 +6151,14 @@
       <c r="F137" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G137" s="2" t="s">
+        <v>730</v>
+      </c>
+      <c r="H137" s="2" t="s">
+        <v>731</v>
+      </c>
+    </row>
+    <row r="138" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
         <v>566</v>
       </c>
@@ -5748,7 +6178,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
         <v>567</v>
       </c>
@@ -5768,7 +6198,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
         <v>572</v>
       </c>
@@ -5788,7 +6218,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
         <v>577</v>
       </c>
@@ -5808,7 +6238,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="142" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
         <v>582</v>
       </c>
@@ -5828,7 +6258,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="143" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
         <v>587</v>
       </c>
@@ -5848,7 +6278,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="144" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
         <v>592</v>
       </c>
@@ -5968,7 +6398,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="150" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
         <v>602</v>
       </c>
@@ -5986,6 +6416,12 @@
       </c>
       <c r="F150" t="s">
         <v>17</v>
+      </c>
+      <c r="G150" s="2" t="s">
+        <v>744</v>
+      </c>
+      <c r="H150" s="2" t="s">
+        <v>745</v>
       </c>
     </row>
     <row r="151" spans="1:8" x14ac:dyDescent="0.3">
@@ -6194,7 +6630,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="161" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
         <v>625</v>
       </c>
@@ -6214,7 +6650,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="162" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
         <v>627</v>
       </c>
@@ -6234,7 +6670,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="163" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
         <v>629</v>
       </c>
@@ -6254,7 +6690,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="164" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
         <v>630</v>
       </c>
@@ -6274,7 +6710,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="165" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A165" t="s">
         <v>635</v>
       </c>
@@ -6294,7 +6730,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="166" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A166" t="s">
         <v>636</v>
       </c>
@@ -6314,7 +6750,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="167" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
         <v>638</v>
       </c>
@@ -6334,7 +6770,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="168" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A168" t="s">
         <v>642</v>
       </c>
@@ -6354,7 +6790,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="169" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A169" t="s">
         <v>644</v>
       </c>
@@ -6373,8 +6809,14 @@
       <c r="F169" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="170" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G169" s="2" t="s">
+        <v>740</v>
+      </c>
+      <c r="H169" s="2" t="s">
+        <v>741</v>
+      </c>
+    </row>
+    <row r="170" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A170" t="s">
         <v>645</v>
       </c>
@@ -6394,7 +6836,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="171" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A171" t="s">
         <v>648</v>
       </c>
@@ -6414,7 +6856,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="172" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A172" t="s">
         <v>650</v>
       </c>
@@ -6434,7 +6876,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="173" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A173" t="s">
         <v>651</v>
       </c>
@@ -6454,7 +6896,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="174" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A174" t="s">
         <v>656</v>
       </c>

</xml_diff>

<commit_message>
feat: add customize quiz mechanic
</commit_message>
<xml_diff>
--- a/raw_csv_quiz/Quiz_Week04.xlsx
+++ b/raw_csv_quiz/Quiz_Week04.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\LearningHub\ai-2y-journey\06-other\flashcard-app\raw_csv_quiz\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{082AE168-3A82-48AC-9FC8-71ED1EF34BDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE6976CA-1355-4D82-BAD5-74352FE66510}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1132" uniqueCount="746">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1133" uniqueCount="747">
   <si>
     <t>Question</t>
   </si>
@@ -2815,6 +2815,13 @@
 AWS WAF (Option C): This is the Bulletproof Glass on the display cases. It's a tool you put in place to stop specific types of theft (web exploits).
 AWS Shield Advanced (The Answer): This is like having a Private Security Firm on retainer. Because you pay for the premium service, you get access to a Rapid Response SWAT Team (the DRT) that will rush to your store during a complex heist to personally fight off the attackers and help you fix the glass. (This Answer)
 Key Exam Keyword: Whenever a question asks about the "DDoS Response Team (DRT)" or "Shield Response Team (SRT)," the answer must include AWS Shield Advanced.</t>
+  </si>
+  <si>
+    <t>B. AWS Secrets Manager.
+While several AWS services deal with security and encryption, AWS Secrets Manager is specifically designed for the lifecycle management of sensitive credentials like database passwords.
+SSM Parameter Store -&gt; Configuration data, feature flags, AMI IDs.
+AWS KMS -&gt; Managing encryption keys (CMKs).
+AWS ACM -&gt; SSL/TLS Certificates for websites.</t>
   </si>
 </sst>
 </file>
@@ -6092,7 +6099,7 @@
         <v>729</v>
       </c>
     </row>
-    <row r="135" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
         <v>553</v>
       </c>
@@ -6110,6 +6117,9 @@
       </c>
       <c r="F135" t="s">
         <v>11</v>
+      </c>
+      <c r="G135" s="2" t="s">
+        <v>746</v>
       </c>
     </row>
     <row r="136" spans="1:8" x14ac:dyDescent="0.3">

</xml_diff>